<commit_message>
52th commit/I am going to uploade two day data
</commit_message>
<xml_diff>
--- a/12617679.xlsx
+++ b/12617679.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD142F85-8424-40AE-92D1-61CB424216A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BDE3F9C-D4EB-4DF9-8ECF-A293C01F87D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="81">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -272,6 +272,12 @@
   </si>
   <si>
     <t>today I am complete analytical CA and I am very happy .</t>
+  </si>
+  <si>
+    <t>In this day I am going to visiti golden temple in amritsar</t>
+  </si>
+  <si>
+    <t>I am return this day .</t>
   </si>
 </sst>
 </file>
@@ -3442,49 +3448,97 @@
         <v>68</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A58" s="13"/>
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="14"/>
-      <c r="F58" s="14"/>
-      <c r="G58" s="14"/>
-      <c r="H58" s="14"/>
-      <c r="I58" s="15" t="str">
+    <row r="58" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+      <c r="A58" s="13">
+        <v>46296</v>
+      </c>
+      <c r="B58" s="14">
+        <v>400</v>
+      </c>
+      <c r="C58" s="14">
+        <v>30</v>
+      </c>
+      <c r="D58" s="14">
+        <v>0</v>
+      </c>
+      <c r="E58" s="14">
+        <v>0</v>
+      </c>
+      <c r="F58" s="14">
+        <v>0</v>
+      </c>
+      <c r="G58" s="14">
+        <v>0</v>
+      </c>
+      <c r="H58" s="14">
+        <v>600</v>
+      </c>
+      <c r="I58" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J58" s="15" t="str">
+        <v>1030</v>
+      </c>
+      <c r="J58" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K58" s="16"/>
-      <c r="L58" s="16"/>
-      <c r="M58" s="16"/>
-      <c r="N58" s="17"/>
+        <v>410</v>
+      </c>
+      <c r="K58" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L58" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="M58" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N58" s="17" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A59" s="13"/>
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="14"/>
-      <c r="F59" s="14"/>
-      <c r="G59" s="14"/>
-      <c r="H59" s="14"/>
-      <c r="I59" s="15" t="str">
+      <c r="A59" s="13">
+        <v>46297</v>
+      </c>
+      <c r="B59" s="14">
+        <v>560</v>
+      </c>
+      <c r="C59" s="14">
+        <v>45</v>
+      </c>
+      <c r="D59" s="14">
+        <v>0</v>
+      </c>
+      <c r="E59" s="14">
+        <v>0</v>
+      </c>
+      <c r="F59" s="14">
+        <v>0</v>
+      </c>
+      <c r="G59" s="14">
+        <v>0</v>
+      </c>
+      <c r="H59" s="14">
+        <v>580</v>
+      </c>
+      <c r="I59" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J59" s="15" t="str">
+        <v>1185</v>
+      </c>
+      <c r="J59" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K59" s="16"/>
-      <c r="L59" s="16"/>
-      <c r="M59" s="16"/>
-      <c r="N59" s="17"/>
+        <v>255</v>
+      </c>
+      <c r="K59" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L59" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M59" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="N59" s="17" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A60" s="13"/>

</xml_diff>